<commit_message>
Adiciona data-base personalizada no gráfico e traz de volta datas de divulgação de resultado
</commit_message>
<xml_diff>
--- a/valuations/AAPL.xlsx
+++ b/valuations/AAPL.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Technology / Consumer Electronics | As of 03/07/2026 | Valores em USD, exceto preço por ação</t>
+          <t>Technology / Consumer Electronics | Gerado em 04/07/2026 | Valores em USD, exceto preço por ação</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>113.6669603452093</v>
+        <v>111.5422166991194</v>
       </c>
     </row>
     <row r="7">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>0.04372000217437744</v>
+        <v>0.0449</v>
       </c>
     </row>
     <row r="14">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>0.08965780217437744</v>
+        <v>0.0908378</v>
       </c>
     </row>
     <row r="16">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>0.0884286213142263</v>
+        <v>0.0895834842738592</v>
       </c>
     </row>
     <row r="24">
@@ -746,311 +746,335 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Crescimento de receita — ano 1 (consenso)</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>0.075</v>
+          <t>↳ período fiscal do documento (10-K/10-Q)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Crescimento na perpetuidade (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>0.025</v>
+          <t>↳ dados buscados do yfinance em</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Margem EBIT (média histórica)</t>
+          <t>Crescimento de receita — ano 1 (consenso)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>0.3174051131633372</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>D&amp;A (% da receita, média histórica)</t>
+          <t>Crescimento na perpetuidade (Gordon Growth)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>0.02868889663320831</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>CapEx ano 1 (guidance pública / histórico)</t>
+          <t>Margem EBIT (média histórica)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>-0.03364082650704896</v>
+        <v>0.3174051131633372</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>CapEx normalizado (média histórica)</t>
+          <t>D&amp;A (% da receita, média histórica)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>-0.02735602098481622</v>
+        <v>0.02868889663320831</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
+          <t>CapEx ano 1 (guidance pública / histórico)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>-0.03364082650704896</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>CapEx normalizado (média histórica)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t>Variação de capital de giro (% da receita)</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="B35" s="7" t="n">
         <v>-0.02536807217015623</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>PROJEÇÃO DE FLUXO DE CAIXA (FCFF)</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Receita</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>CapEx (% receita)</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>Valor Presente do FCFF</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B37" s="16" t="n">
-        <v>447373075000</v>
-      </c>
-      <c r="C37" s="17" t="n">
-        <v>-0.03364082650704896</v>
-      </c>
-      <c r="D37" s="16" t="n">
-        <v>100246603285</v>
-      </c>
-      <c r="E37" s="16" t="n">
-        <v>92102138185</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B38" s="16" t="n">
-        <v>475333892188</v>
-      </c>
-      <c r="C38" s="17" t="n">
-        <v>-0.02735602098481622</v>
-      </c>
-      <c r="D38" s="16" t="n">
-        <v>109499397061</v>
-      </c>
-      <c r="E38" s="16" t="n">
-        <v>92429759048</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B39" s="16" t="n">
-        <v>499100586797</v>
+        <v>447373075000</v>
       </c>
       <c r="C39" s="17" t="n">
-        <v>-0.02735602098481622</v>
+        <v>-0.03364082650704896</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>114974366914</v>
+        <v>100246603285</v>
       </c>
       <c r="E39" s="16" t="n">
-        <v>89166386385</v>
+        <v>92004517994</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B40" s="16" t="n">
-        <v>517816858802</v>
+        <v>475333892188</v>
       </c>
       <c r="C40" s="17" t="n">
         <v>-0.02735602098481622</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>119285905673</v>
+        <v>109499397061</v>
       </c>
       <c r="E40" s="16" t="n">
-        <v>84994205465</v>
+        <v>92233928004</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B41" s="16" t="n">
-        <v>530762280272</v>
+        <v>499100586797</v>
       </c>
       <c r="C41" s="17" t="n">
         <v>-0.02735602098481622</v>
       </c>
       <c r="D41" s="16" t="n">
+        <v>114974366914</v>
+      </c>
+      <c r="E41" s="16" t="n">
+        <v>88883161136</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B42" s="16" t="n">
+        <v>517816858802</v>
+      </c>
+      <c r="C42" s="17" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>119285905673</v>
+      </c>
+      <c r="E42" s="16" t="n">
+        <v>84634432340</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B43" s="16" t="n">
+        <v>530762280272</v>
+      </c>
+      <c r="C43" s="17" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+      <c r="D43" s="16" t="n">
         <v>122268053315</v>
       </c>
-      <c r="E41" s="16" t="n">
-        <v>80041133516</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Soma dos VPs dos FCFF projetados</t>
-        </is>
-      </c>
-      <c r="B43" s="11">
-        <f>SUM(E37:E41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Valor terminal (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="n">
-        <v>1975839172464.143</v>
+      <c r="E43" s="16" t="n">
+        <v>79617848839</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Valor presente do valor terminal</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="n">
-        <v>1293456489428.469</v>
+          <t>Soma dos VPs dos FCFF projetados</t>
+        </is>
+      </c>
+      <c r="B45" s="11">
+        <f>SUM(E39:E43)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="inlineStr">
-        <is>
-          <t>Valor da empresa (Enterprise Value)</t>
-        </is>
-      </c>
-      <c r="B46" s="18">
-        <f>B43+B45</f>
-        <v/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Valor terminal (Gordon Growth)</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="n">
+        <v>1940507794788.78</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>(-) Dívida líquida</t>
+          <t>Valor presente do valor terminal</t>
         </is>
       </c>
       <c r="B47" s="11" t="n">
-        <v>62723000000</v>
+        <v>1263609357375.074</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>Valor do equity</t>
+          <t>Valor da empresa (Enterprise Value)</t>
         </is>
       </c>
       <c r="B48" s="18">
-        <f>B46-B47</f>
+        <f>B45+B47</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Ações em circulação</t>
-        </is>
-      </c>
-      <c r="B49" s="19" t="n">
-        <v>14687356000</v>
+          <t>(-) Dívida líquida</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="n">
+        <v>62723000000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
+          <t>Valor do equity</t>
+        </is>
+      </c>
+      <c r="B50" s="18">
+        <f>B48-B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Ações em circulação</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="n">
+        <v>14687356000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
           <t>Preço-alvo por ação (=Valor do equity / Ações)</t>
         </is>
       </c>
-      <c r="B50" s="20">
-        <f>B48/B49</f>
+      <c r="B52" s="20">
+        <f>B50/B51</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="21" t="inlineStr">
-        <is>
-          <t>• Fonte dos dados: pipeline próprio (yfinance -&gt; SQLite via src/data_fetch.py). Cálculo do DCF: src/dcf.py (versionado no Git).</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="21" t="inlineStr">
-        <is>
-          <t>• CapEx: parte da guidance pública de investimento (quando disponível) e normaliza rápido (config.ANOS_FADE_CAPEX=2 anos) para a média histórica — reflete o pico atual de investimento em IA sem assumir uma trajetória de longo prazo que não temos base para prever.</t>
-        </is>
-      </c>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
+        <is>
+          <t>• Fonte dos dados: pipeline próprio (yfinance -&gt; SQLite via src/data_fetch.py). Cálculo do DCF: src/dcf.py (versionado no Git).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>• CapEx: parte da guidance pública de investimento (quando disponível) e normaliza rápido (config.ANOS_FADE_CAPEX=2 anos) para a média histórica — reflete o pico atual de investimento em IA sem assumir uma trajetória de longo prazo que não temos base para prever.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>• Limitação conhecida: DCF simples de horizonte curto tende a subestimar mega caps de crescimento (não captura opcionalidade/crescimento além do período explícito). Ver comps_analysis.xlsx para cross-check via múltiplos de mercado.</t>
         </is>
@@ -1059,15 +1083,15 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A56:G56"/>
     <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A57:G57"/>
     <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona atalho de duplo-clique para atualizar dados sem terminal
</commit_message>
<xml_diff>
--- a/valuations/AAPL.xlsx
+++ b/valuations/AAPL.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -541,557 +541,577 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Preço-alvo (DCF)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>111.5422166991194</v>
+          <t>↳ preço de fechamento de</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>Preço-alvo (DCF)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>111.6307106314984</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>Upside / Downside</t>
         </is>
       </c>
-      <c r="B7" s="7">
-        <f>(B6/B5)-1</f>
+      <c r="B8" s="7">
+        <f>(B7/B5)-1</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Recomendação</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Venda</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Threshold Compra / Venda</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>&gt;15% / &lt;-15%</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>WACC (CAPM)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1.086</v>
-      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Taxa livre de risco (Treasury 10Y)</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n">
-        <v>0.0449</v>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1.086</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Prêmio de risco de mercado (ERP, Damodaran)</t>
+          <t>Taxa livre de risco (Treasury 10Y)</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>0.0423</v>
+        <v>0.04484999656677246</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Custo do capital próprio (CAPM)</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="n">
-        <v>0.0908378</v>
-      </c>
+          <t>↳ fonte: ao vivo (pregão de 2026-07-02)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Dívida total</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n">
-        <v>98657000000</v>
+          <t>Prêmio de risco de mercado (ERP, Damodaran)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0.0423</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Custo da dívida pré-imposto (Desp. Juros / Dívida)</t>
+          <t>Custo do capital próprio (CAPM)</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>0.03986539221748077</v>
+        <v>0.09078779656677247</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Taxa de imposto efetiva</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>0.1985059374988801</v>
+          <t>Dívida total</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>98657000000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Custo da dívida pós-imposto</t>
+          <t>Custo da dívida pré-imposto (Desp. Juros / Dívida)</t>
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>0.03195187516158919</v>
+        <v>0.03986539221748077</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Valor de mercado do equity</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="n">
-        <v>4532958920704</v>
+          <t>Taxa de imposto efetiva</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.1985059374988801</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Custo da dívida pós-imposto</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>0.03195187516158919</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Valor de mercado do equity</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>4532958920704</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Peso equity / Peso dívida</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>97.9% / 2.1%</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
-        <v>0.0895834842738592</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="B24" s="13" t="n">
+        <v>0.08953454595241908</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>PREMISSAS DE PROJEÇÃO</t>
         </is>
       </c>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Horizonte de projeção explícita</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>5 anos</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Receita base (mais recente)</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="n">
-        <v>416161000000</v>
-      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>↳ período fiscal do documento (10-K/10-Q)</t>
+          <t>Horizonte de projeção explícita</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>5 anos</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>↳ dados buscados do yfinance em</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
+          <t>Receita base (mais recente)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>416161000000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Crescimento de receita — ano 1 (consenso)</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>0.075</v>
+          <t>↳ período fiscal do documento (10-K/10-Q)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Crescimento na perpetuidade (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>0.025</v>
+          <t>↳ dados buscados do yfinance em</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Margem EBIT (média histórica)</t>
+          <t>Crescimento de receita — ano 1 (consenso)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>0.3174051131633372</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>D&amp;A (% da receita, média histórica)</t>
+          <t>Crescimento na perpetuidade (Gordon Growth)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>0.02868889663320831</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>CapEx ano 1 (guidance pública / histórico)</t>
+          <t>Margem EBIT (média histórica)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>-0.03364082650704896</v>
+        <v>0.3174051131633372</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>CapEx normalizado (média histórica)</t>
+          <t>D&amp;A (% da receita, média histórica)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>-0.02735602098481622</v>
+        <v>0.02868889663320831</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
+          <t>CapEx ano 1 (guidance pública / histórico)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>-0.03364082650704896</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>CapEx normalizado (média histórica)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>Variação de capital de giro (% da receita)</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B37" s="7" t="n">
         <v>-0.02536807217015623</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>PROJEÇÃO DE FLUXO DE CAIXA (FCFF)</t>
         </is>
       </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="4" t="n"/>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>Receita</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>CapEx (% receita)</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
+      <c r="E40" s="14" t="inlineStr">
         <is>
           <t>Valor Presente do FCFF</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" s="16" t="n">
-        <v>447373075000</v>
-      </c>
-      <c r="C39" s="17" t="n">
-        <v>-0.03364082650704896</v>
-      </c>
-      <c r="D39" s="16" t="n">
-        <v>100246603285</v>
-      </c>
-      <c r="E39" s="16" t="n">
-        <v>92004517994</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B40" s="16" t="n">
-        <v>475333892188</v>
-      </c>
-      <c r="C40" s="17" t="n">
-        <v>-0.02735602098481622</v>
-      </c>
-      <c r="D40" s="16" t="n">
-        <v>109499397061</v>
-      </c>
-      <c r="E40" s="16" t="n">
-        <v>92233928004</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B41" s="16" t="n">
-        <v>499100586797</v>
+        <v>447373075000</v>
       </c>
       <c r="C41" s="17" t="n">
-        <v>-0.02735602098481622</v>
+        <v>-0.03364082650704896</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>114974366914</v>
+        <v>100246603285</v>
       </c>
       <c r="E41" s="16" t="n">
-        <v>88883161136</v>
+        <v>92008650536</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B42" s="16" t="n">
-        <v>517816858802</v>
+        <v>475333892188</v>
       </c>
       <c r="C42" s="17" t="n">
         <v>-0.02735602098481622</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>119285905673</v>
+        <v>109499397061</v>
       </c>
       <c r="E42" s="16" t="n">
-        <v>84634432340</v>
+        <v>92242213882</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B43" s="16" t="n">
-        <v>530762280272</v>
+        <v>499100586797</v>
       </c>
       <c r="C43" s="17" t="n">
         <v>-0.02735602098481622</v>
       </c>
       <c r="D43" s="16" t="n">
+        <v>114974366914</v>
+      </c>
+      <c r="E43" s="16" t="n">
+        <v>88895138695</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="16" t="n">
+        <v>517816858802</v>
+      </c>
+      <c r="C44" s="17" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>119285905673</v>
+      </c>
+      <c r="E44" s="16" t="n">
+        <v>84649639370</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B45" s="16" t="n">
+        <v>530762280272</v>
+      </c>
+      <c r="C45" s="17" t="n">
+        <v>-0.02735602098481622</v>
+      </c>
+      <c r="D45" s="16" t="n">
         <v>122268053315</v>
       </c>
-      <c r="E43" s="16" t="n">
-        <v>79617848839</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Soma dos VPs dos FCFF projetados</t>
-        </is>
-      </c>
-      <c r="B45" s="11">
-        <f>SUM(E39:E43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Valor terminal (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="n">
-        <v>1940507794788.78</v>
+      <c r="E45" s="16" t="n">
+        <v>79635731310</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Valor presente do valor terminal</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="n">
-        <v>1263609357375.074</v>
+          <t>Soma dos VPs dos FCFF projetados</t>
+        </is>
+      </c>
+      <c r="B47" s="11">
+        <f>SUM(E41:E45)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="inlineStr">
-        <is>
-          <t>Valor da empresa (Enterprise Value)</t>
-        </is>
-      </c>
-      <c r="B48" s="18">
-        <f>B45+B47</f>
-        <v/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Valor terminal (Gordon Growth)</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>1941979335229.902</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>(-) Dívida líquida</t>
+          <t>Valor presente do valor terminal</t>
         </is>
       </c>
       <c r="B49" s="11" t="n">
-        <v>62723000000</v>
+        <v>1264851613784.999</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>Valor do equity</t>
+          <t>Valor da empresa (Enterprise Value)</t>
         </is>
       </c>
       <c r="B50" s="18">
-        <f>B48-B49</f>
+        <f>B47+B49</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Ações em circulação</t>
-        </is>
-      </c>
-      <c r="B51" s="19" t="n">
-        <v>14687356000</v>
+          <t>(-) Dívida líquida</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="n">
+        <v>62723000000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
+          <t>Valor do equity</t>
+        </is>
+      </c>
+      <c r="B52" s="18">
+        <f>B50-B51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Ações em circulação</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n">
+        <v>14687356000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
           <t>Preço-alvo por ação (=Valor do equity / Ações)</t>
         </is>
       </c>
-      <c r="B52" s="20">
-        <f>B50/B51</f>
+      <c r="B54" s="20">
+        <f>B52/B53</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>NOTAS</t>
         </is>
       </c>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="21" t="inlineStr">
-        <is>
-          <t>• Fonte dos dados: pipeline próprio (yfinance -&gt; SQLite via src/data_fetch.py). Cálculo do DCF: src/dcf.py (versionado no Git).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="21" t="inlineStr">
-        <is>
-          <t>• CapEx: parte da guidance pública de investimento (quando disponível) e normaliza rápido (config.ANOS_FADE_CAPEX=2 anos) para a média histórica — reflete o pico atual de investimento em IA sem assumir uma trajetória de longo prazo que não temos base para prever.</t>
-        </is>
-      </c>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="21" t="inlineStr">
         <is>
+          <t>• Fonte dos dados: pipeline próprio (yfinance -&gt; SQLite via src/data_fetch.py). Cálculo do DCF: src/dcf.py (versionado no Git).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="21" t="inlineStr">
+        <is>
+          <t>• CapEx: parte da guidance pública de investimento (quando disponível) e normaliza rápido (config.ANOS_FADE_CAPEX=2 anos) para a média histórica — reflete o pico atual de investimento em IA sem assumir uma trajetória de longo prazo que não temos base para prever.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="21" t="inlineStr">
+        <is>
           <t>• Limitação conhecida: DCF simples de horizonte curto tende a subestimar mega caps de crescimento (não captura opcionalidade/crescimento além do período explícito). Ver comps_analysis.xlsx para cross-check via múltiplos de mercado.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A56:G56"/>
-    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A59:G59"/>
     <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>